<commit_message>
new calibration and fullscreen window update
</commit_message>
<xml_diff>
--- a/internetconfig.xlsx
+++ b/internetconfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeAMK_Vision_Project-master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B26777F0-EAF9-487E-BF08-438F4520A316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79E9130B-F570-413C-9088-2E0B1018C25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{E7932B6A-9915-4B30-90BC-D46ABED7F28F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E7932B6A-9915-4B30-90BC-D46ABED7F28F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
   <si>
     <t>Advanced EEE</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>Not Speed Down</t>
+  </si>
+  <si>
+    <t>maximum if able</t>
   </si>
 </sst>
 </file>
@@ -556,15 +559,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F23BE8C-6041-4179-A2F8-6B282F65598F}">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.7265625" style="1"/>
+    <col min="3" max="3" width="14" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -572,7 +576,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -580,7 +584,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -588,7 +592,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -596,7 +600,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -604,7 +608,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -612,7 +616,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -620,7 +624,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -628,7 +632,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -636,7 +640,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -644,7 +648,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -652,7 +656,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -660,7 +664,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
@@ -668,7 +672,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -676,7 +680,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -684,12 +688,15 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="1">
         <v>512</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>